<commit_message>
Weekly logs and research logs
</commit_message>
<xml_diff>
--- a/Evidence Handling/Olivia Evidence/Evidence Handling Record.xlsx
+++ b/Evidence Handling/Olivia Evidence/Evidence Handling Record.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3d87909e21b199fc/Documents/BHB-Capstone/Evidence Handling/Olivia Evidence/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="8" documentId="8_{0AD82C83-FB65-4B68-B458-35F57E22243A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{947B9121-5CD0-4259-87D9-3D2A9150CEE9}"/>
+  <xr:revisionPtr revIDLastSave="9" documentId="8_{0AD82C83-FB65-4B68-B458-35F57E22243A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B76C97A9-2294-4E19-88BC-8FBFAA5C0A40}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{4B523841-F448-4F74-9155-C94C48BB4A19}"/>
+    <workbookView xWindow="2410" yWindow="830" windowWidth="16790" windowHeight="8300" xr2:uid="{4B523841-F448-4F74-9155-C94C48BB4A19}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="19">
   <si>
     <t>Evidence / File Type</t>
   </si>
@@ -96,9 +96,6 @@
   </si>
   <si>
     <t>/home/pcadmin/Desktop/Artefacts/Evidence/THREE.dd</t>
-  </si>
-  <si>
-    <t>e_002</t>
   </si>
 </sst>
 </file>
@@ -160,6 +157,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -479,7 +480,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{96D9203E-1CA1-4B1F-902E-282449A7789A}">
-  <dimension ref="B3:H6"/>
+  <dimension ref="B3:H5"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="19.08984375" customWidth="1"/>
@@ -561,11 +562,6 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="C6" t="s">
-        <v>19</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Added evidence02.pcapng wireshark report, evidence handling and updated report tracking spreadsheet
</commit_message>
<xml_diff>
--- a/Evidence Handling/Olivia Evidence/Evidence Handling Record.xlsx
+++ b/Evidence Handling/Olivia Evidence/Evidence Handling Record.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3d87909e21b199fc/Documents/BHB-Capstone/Evidence Handling/Olivia Evidence/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="9" documentId="8_{0AD82C83-FB65-4B68-B458-35F57E22243A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B76C97A9-2294-4E19-88BC-8FBFAA5C0A40}"/>
+  <xr:revisionPtr revIDLastSave="15" documentId="8_{0AD82C83-FB65-4B68-B458-35F57E22243A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{83039DD6-D191-4AB6-B401-B2044B2C907D}"/>
   <bookViews>
-    <workbookView xWindow="2410" yWindow="830" windowWidth="16790" windowHeight="8300" xr2:uid="{4B523841-F448-4F74-9155-C94C48BB4A19}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{4B523841-F448-4F74-9155-C94C48BB4A19}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="23">
   <si>
     <t>Evidence / File Type</t>
   </si>
@@ -96,6 +96,18 @@
   </si>
   <si>
     <t>/home/pcadmin/Desktop/Artefacts/Evidence/THREE.dd</t>
+  </si>
+  <si>
+    <t>evidence02.pcapng</t>
+  </si>
+  <si>
+    <t>/home/pcadmin/Desktop/Artefacts/Evidence/evidence02.pcapng</t>
+  </si>
+  <si>
+    <t>pcapng</t>
+  </si>
+  <si>
+    <t>7516e76851baacc0587ee4f0bff397f9</t>
   </si>
 </sst>
 </file>
@@ -139,9 +151,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -480,7 +493,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{96D9203E-1CA1-4B1F-902E-282449A7789A}">
-  <dimension ref="B3:H5"/>
+  <dimension ref="B3:H6"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="19.08984375" customWidth="1"/>
@@ -562,6 +575,23 @@
         <v>17</v>
       </c>
     </row>
+    <row r="6" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="D6" t="s">
+        <v>19</v>
+      </c>
+      <c r="E6" t="s">
+        <v>20</v>
+      </c>
+      <c r="F6" t="s">
+        <v>8</v>
+      </c>
+      <c r="G6" t="s">
+        <v>21</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>22</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>